<commit_message>
Add batch Excel write tool to handle large text content and prevent JSON parsing errors
</commit_message>
<xml_diff>
--- a/output/测试合同-HT-2025-001.xlsx
+++ b/output/测试合同-HT-2025-001.xlsx
@@ -143,21 +143,21 @@
     <t>购货方</t>
   </si>
   <si>
+    <t>供货方</t>
+  </si>
+  <si>
     <t>签（公）证意见：</t>
   </si>
   <si>
-    <t>供货方</t>
-  </si>
-  <si>
     <t>单位名称（盖章）：湖南陶润会文化传播有限公司工会委员会</t>
   </si>
   <si>
+    <t>单位名称（盖章）：醴陵市时尚灯饰经营部</t>
+  </si>
+  <si>
     <t>经办人：</t>
   </si>
   <si>
-    <t>单位名称（盖章）：醴陵市时尚灯饰经营部</t>
-  </si>
-  <si>
     <t>法定代表人：</t>
   </si>
   <si>
@@ -170,31 +170,31 @@
     <t>电    话：</t>
   </si>
   <si>
+    <t>电    话：15273352244</t>
+  </si>
+  <si>
     <t>签（公）证机关（章）</t>
   </si>
   <si>
-    <t>电    话：15273352244</t>
-  </si>
-  <si>
     <t>传    真：</t>
   </si>
   <si>
     <t>开户行：</t>
   </si>
   <si>
+    <t>开户行：中国农业银行醴陵市城东支行</t>
+  </si>
+  <si>
     <t xml:space="preserve">         年    月    日</t>
   </si>
   <si>
-    <t>开户行：中国农业银行醴陵市城东支行</t>
-  </si>
-  <si>
     <t>账    号：</t>
   </si>
   <si>
+    <t>账    号：6228481109443211071</t>
+  </si>
+  <si>
     <t>注：除国家另有规定外，签（公）证实行自愿原则</t>
-  </si>
-  <si>
-    <t>账    号：6228481109443211071</t>
   </si>
 </sst>
 </file>
@@ -577,78 +577,78 @@
       <c r="A24" t="s" s="5">
         <v>42</v>
       </c>
-      <c r="C24" t="s" s="5">
+      <c r="D24" t="s" s="5">
         <v>43</v>
       </c>
-      <c r="F24" t="s" s="5">
+      <c r="G24" t="s" s="5">
         <v>44</v>
       </c>
     </row>
     <row r="25" ht="19.0" customHeight="true">
-      <c r="A25" t="s" s="5">
+      <c r="A25" t="s" s="4">
         <v>45</v>
       </c>
-      <c r="C25" t="s" s="5">
+      <c r="D25" t="s" s="4">
         <v>46</v>
       </c>
-      <c r="F25" t="s" s="5">
+      <c r="G25" t="s" s="4">
         <v>47</v>
       </c>
     </row>
     <row r="26" ht="19.0" customHeight="true">
-      <c r="A26" t="s" s="5">
+      <c r="A26" t="s" s="4">
         <v>48</v>
       </c>
-      <c r="F26" t="s" s="5">
+      <c r="D26" t="s" s="4">
         <v>49</v>
       </c>
     </row>
     <row r="27" ht="19.0" customHeight="true">
-      <c r="A27" t="s" s="5">
+      <c r="A27" t="s" s="4">
         <v>50</v>
       </c>
-      <c r="F27" t="s" s="5">
+      <c r="D27" t="s" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="28" ht="19.0" customHeight="true">
-      <c r="A28" t="s" s="5">
+      <c r="A28" t="s" s="4">
         <v>51</v>
       </c>
-      <c r="C28" t="s" s="5">
+      <c r="D28" t="s" s="4">
         <v>52</v>
       </c>
-      <c r="F28" t="s" s="5">
+      <c r="G28" t="s" s="4">
         <v>53</v>
       </c>
     </row>
     <row r="29" ht="19.0" customHeight="true">
-      <c r="A29" t="s" s="5">
+      <c r="A29" t="s" s="4">
         <v>54</v>
       </c>
-      <c r="F29" t="s" s="5">
+      <c r="D29" t="s" s="4">
         <v>54</v>
       </c>
     </row>
     <row r="30" ht="19.0" customHeight="true">
-      <c r="A30" t="s" s="5">
+      <c r="A30" t="s" s="4">
         <v>55</v>
       </c>
-      <c r="C30" t="s" s="5">
+      <c r="D30" t="s" s="4">
         <v>56</v>
       </c>
-      <c r="F30" t="s" s="5">
+      <c r="G30" t="s" s="4">
         <v>57</v>
       </c>
     </row>
     <row r="31" ht="19.0" customHeight="true">
-      <c r="A31" t="s" s="5">
+      <c r="A31" t="s" s="4">
         <v>58</v>
       </c>
-      <c r="C31" t="s" s="5">
+      <c r="D31" t="s" s="4">
         <v>59</v>
       </c>
-      <c r="F31" t="s" s="5">
+      <c r="G31" t="s" s="4">
         <v>60</v>
       </c>
     </row>
@@ -675,27 +675,27 @@
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:H31"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix contract clause updates by supporting custom clauses in both create and update methods
</commit_message>
<xml_diff>
--- a/output/测试合同-HT-2025-001.xlsx
+++ b/output/测试合同-HT-2025-001.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="61">
   <si>
     <t>湖南陶润会文化传播有限公司工会委员会</t>
   </si>
@@ -202,13 +202,67 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="17">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="16.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="10.0"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="10.0"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="16.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="10.0"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="10.0"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="16.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="10.0"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="10.0"/>
     </font>
     <font>
       <name val="宋体"/>
@@ -277,7 +331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -292,6 +346,51 @@
       <alignment horizontal="left" vertical="center" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -303,14 +402,14 @@
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="14.0" customWidth="true"/>
-    <col min="2" max="2" width="23.0" customWidth="true"/>
-    <col min="3" max="3" width="28.0" customWidth="true"/>
-    <col min="4" max="4" width="10.0" customWidth="true"/>
-    <col min="5" max="5" width="8.0" customWidth="true"/>
-    <col min="6" max="6" width="10.0" customWidth="true"/>
-    <col min="7" max="7" width="15.0" customWidth="true"/>
-    <col min="8" max="8" width="16.0" customWidth="true"/>
+    <col min="1" max="1" customWidth="true" width="14.0"/>
+    <col min="2" max="2" customWidth="true" width="23.0"/>
+    <col min="3" max="3" customWidth="true" width="28.0"/>
+    <col min="4" max="4" customWidth="true" width="10.0"/>
+    <col min="5" max="5" customWidth="true" width="8.0"/>
+    <col min="6" max="6" customWidth="true" width="10.0"/>
+    <col min="7" max="7" customWidth="true" width="15.0"/>
+    <col min="8" max="8" customWidth="true" width="16.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.0" customHeight="true">
@@ -391,111 +490,111 @@
       </c>
     </row>
     <row r="8" ht="19.0" customHeight="true">
-      <c r="A8" t="s" s="3">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s" s="3">
+      <c r="A8" t="s" s="18">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="C8" t="s" s="3">
+      <c r="C8" t="s" s="18">
         <v>22</v>
       </c>
-      <c r="D8" t="n" s="3">
+      <c r="D8" t="n" s="18">
         <v>64.0</v>
       </c>
-      <c r="E8" t="s" s="3">
+      <c r="E8" t="s" s="18">
         <v>23</v>
       </c>
-      <c r="F8" t="n" s="3">
+      <c r="F8" t="n" s="18">
         <v>23.0</v>
       </c>
-      <c r="G8" t="n" s="3">
+      <c r="G8" t="n" s="18">
         <v>1472.0</v>
       </c>
-      <c r="H8" t="s" s="3">
+      <c r="H8" t="s" s="18">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="19.0" customHeight="true">
-      <c r="A9" t="s" s="3">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s" s="3">
+      <c r="A9" t="s" s="18">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="C9" t="s" s="3">
+      <c r="C9" t="s" s="18">
         <v>24</v>
       </c>
-      <c r="D9" t="n" s="3">
+      <c r="D9" t="n" s="18">
         <v>32.0</v>
       </c>
-      <c r="E9" t="s" s="3">
+      <c r="E9" t="s" s="18">
         <v>25</v>
       </c>
-      <c r="F9" t="n" s="3">
+      <c r="F9" t="n" s="18">
         <v>76.0</v>
       </c>
-      <c r="G9" t="n" s="3">
+      <c r="G9" t="n" s="18">
         <v>2432.0</v>
       </c>
-      <c r="H9" t="s" s="3">
+      <c r="H9" t="s" s="18">
         <v>20</v>
       </c>
     </row>
     <row r="10" ht="19.0" customHeight="true">
-      <c r="A10" t="s" s="3">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s" s="3">
+      <c r="A10" t="s" s="18">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="C10" t="s" s="3">
+      <c r="C10" t="s" s="18">
         <v>26</v>
       </c>
-      <c r="D10" t="n" s="3">
+      <c r="D10" t="n" s="18">
         <v>32.0</v>
       </c>
-      <c r="E10" t="s" s="3">
+      <c r="E10" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F10" t="n" s="3">
+      <c r="F10" t="n" s="18">
         <v>73.0</v>
       </c>
-      <c r="G10" t="n" s="3">
+      <c r="G10" t="n" s="18">
         <v>2336.0</v>
       </c>
-      <c r="H10" t="s" s="3">
+      <c r="H10" t="s" s="18">
         <v>20</v>
       </c>
     </row>
     <row r="11" ht="19.0" customHeight="true">
-      <c r="A11" t="s" s="3">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s" s="3">
+      <c r="A11" t="s" s="18">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="C11" t="s" s="3">
+      <c r="C11" t="s" s="18">
         <v>28</v>
       </c>
-      <c r="D11" t="n" s="3">
+      <c r="D11" t="n" s="18">
         <v>28.0</v>
       </c>
-      <c r="E11" t="s" s="3">
+      <c r="E11" t="s" s="18">
         <v>29</v>
       </c>
-      <c r="F11" t="n" s="3">
+      <c r="F11" t="n" s="18">
         <v>4.0</v>
       </c>
-      <c r="G11" t="n" s="3">
+      <c r="G11" t="n" s="18">
         <v>112.0</v>
       </c>
-      <c r="H11" t="s" s="3">
+      <c r="H11" t="s" s="18">
         <v>20</v>
       </c>
     </row>
     <row r="12" ht="19.0" customHeight="true">
-      <c r="A12" t="s" s="3">
+      <c r="A12" t="s" s="18">
         <v>30</v>
       </c>
       <c r="B12" t="s" s="3">
@@ -504,7 +603,7 @@
       <c r="C12" t="s" s="3">
         <v>20</v>
       </c>
-      <c r="D12" t="n" s="3">
+      <c r="D12" t="n" s="18">
         <v>156.0</v>
       </c>
       <c r="E12" t="s" s="3">
@@ -513,7 +612,7 @@
       <c r="F12" t="s" s="3">
         <v>20</v>
       </c>
-      <c r="G12" t="n" s="3">
+      <c r="G12" t="n" s="18">
         <v>6352.0</v>
       </c>
       <c r="H12" t="s" s="3">
@@ -524,52 +623,52 @@
       <c r="A13" t="s" s="5">
         <v>31</v>
       </c>
-      <c r="B13" t="s" s="5">
+      <c r="B13" t="s" s="20">
         <v>32</v>
       </c>
     </row>
     <row r="14" ht="19.0" customHeight="true">
-      <c r="A14" t="s" s="4">
+      <c r="A14" t="s" s="19">
         <v>33</v>
       </c>
     </row>
     <row r="15" ht="19.0" customHeight="true">
-      <c r="A15" t="s" s="4">
+      <c r="A15" t="s" s="19">
         <v>34</v>
       </c>
     </row>
     <row r="16" ht="19.0" customHeight="true">
-      <c r="A16" t="s" s="4">
+      <c r="A16" t="s" s="19">
         <v>35</v>
       </c>
     </row>
     <row r="17" ht="19.0" customHeight="true">
-      <c r="A17" t="s" s="4">
+      <c r="A17" t="s" s="19">
         <v>36</v>
       </c>
     </row>
     <row r="18" ht="19.0" customHeight="true">
-      <c r="A18" t="s" s="4">
+      <c r="A18" t="s" s="19">
         <v>37</v>
       </c>
     </row>
     <row r="19" ht="19.0" customHeight="true">
-      <c r="A19" t="s" s="4">
+      <c r="A19" t="s" s="19">
         <v>38</v>
       </c>
     </row>
     <row r="20" ht="19.0" customHeight="true">
-      <c r="A20" t="s" s="4">
+      <c r="A20" t="s" s="19">
         <v>39</v>
       </c>
     </row>
     <row r="21" ht="19.0" customHeight="true">
-      <c r="A21" t="s" s="4">
+      <c r="A21" t="s" s="19">
         <v>40</v>
       </c>
     </row>
     <row r="22" ht="19.0" customHeight="true">
-      <c r="A22" t="s" s="4">
+      <c r="A22" t="s" s="19">
         <v>41</v>
       </c>
     </row>

</xml_diff>